<commit_message>
Auto scew complete need to finish tele
</commit_message>
<xml_diff>
--- a/output_data.xlsx
+++ b/output_data.xlsx
@@ -44705,10 +44705,10 @@
         <v>66.66666666666666</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>63.33333333333333</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -44784,7 +44784,7 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>22.5</v>
+        <v>0</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -44939,7 +44939,7 @@
         <v>0</v>
       </c>
       <c r="K16">
-        <v>2.222222222222221</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L16" t="s">
         <v>31</v>
@@ -44977,7 +44977,7 @@
         <v>0</v>
       </c>
       <c r="K17">
-        <v>2.222222222222221</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L17" t="s">
         <v>24</v>
@@ -45316,7 +45316,7 @@
         <v>0</v>
       </c>
       <c r="J26">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -45845,10 +45845,10 @@
         <v>0</v>
       </c>
       <c r="I40">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J40">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K40">
         <v>0</v>
@@ -46304,7 +46304,7 @@
         <v>0</v>
       </c>
       <c r="J52">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="K52">
         <v>0</v>
@@ -46339,7 +46339,7 @@
         <v>0</v>
       </c>
       <c r="I53">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J53">
         <v>0</v>
@@ -46535,7 +46535,7 @@
         <v>0</v>
       </c>
       <c r="K58">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L58" t="s">
         <v>31</v>
@@ -46573,7 +46573,7 @@
         <v>0</v>
       </c>
       <c r="K59">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L59" t="s">
         <v>24</v>
@@ -46646,7 +46646,7 @@
         <v>0</v>
       </c>
       <c r="J61">
-        <v>0</v>
+        <v>16.36363636363636</v>
       </c>
       <c r="K61">
         <v>22.5</v>
@@ -47517,7 +47517,7 @@
         <v>33.33333333333333</v>
       </c>
       <c r="I84">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="J84">
         <v>0</v>
@@ -48207,7 +48207,7 @@
         <v>0</v>
       </c>
       <c r="K102">
-        <v>10</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L102" t="s">
         <v>44</v>
@@ -48245,7 +48245,7 @@
         <v>0</v>
       </c>
       <c r="K103">
-        <v>10</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L103" t="s">
         <v>46</v>
@@ -48280,7 +48280,7 @@
         <v>7.499999999999998</v>
       </c>
       <c r="J104">
-        <v>0</v>
+        <v>16.36363636363636</v>
       </c>
       <c r="K104">
         <v>0</v>
@@ -48508,7 +48508,7 @@
         <v>359.9999999999999</v>
       </c>
       <c r="J110">
-        <v>0</v>
+        <v>255.7894736842105</v>
       </c>
       <c r="K110">
         <v>0</v>
@@ -48587,7 +48587,7 @@
         <v>0</v>
       </c>
       <c r="K112">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L112" t="s">
         <v>31</v>
@@ -48625,7 +48625,7 @@
         <v>0</v>
       </c>
       <c r="K113">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L113" t="s">
         <v>26</v>
@@ -49075,7 +49075,7 @@
         <v>0</v>
       </c>
       <c r="I125">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="J125">
         <v>0</v>
@@ -49347,7 +49347,7 @@
         <v>0</v>
       </c>
       <c r="K132">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L132" t="s">
         <v>31</v>
@@ -49385,7 +49385,7 @@
         <v>0</v>
       </c>
       <c r="K133">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="L133" t="s">
         <v>26</v>
@@ -50025,7 +50025,7 @@
         <v>0</v>
       </c>
       <c r="I150">
-        <v>4.615384615384614</v>
+        <v>0</v>
       </c>
       <c r="J150">
         <v>0</v>
@@ -50636,7 +50636,7 @@
         <v>0</v>
       </c>
       <c r="J166">
-        <v>3.789473684210526</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="K166">
         <v>0</v>
@@ -50785,10 +50785,10 @@
         <v>0</v>
       </c>
       <c r="I170">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J170">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="K170">
         <v>0</v>
@@ -51013,10 +51013,10 @@
         <v>33.33333333333333</v>
       </c>
       <c r="I176">
-        <v>0</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="J176">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K176">
         <v>0</v>
@@ -51358,7 +51358,7 @@
         <v>0</v>
       </c>
       <c r="J185">
-        <v>0</v>
+        <v>89.99999999999999</v>
       </c>
       <c r="K185">
         <v>0</v>
@@ -51507,10 +51507,10 @@
         <v>33.33333333333333</v>
       </c>
       <c r="I189">
-        <v>0</v>
+        <v>16.36363636363636</v>
       </c>
       <c r="J189">
-        <v>0</v>
+        <v>16.36363636363636</v>
       </c>
       <c r="K189">
         <v>0</v>

</xml_diff>